<commit_message>
Updated examples for Compositions
</commit_message>
<xml_diff>
--- a/input/assets/Mappings/M11 to FHIR Mapping 01.xlsx
+++ b/input/assets/Mappings/M11 to FHIR Mapping 01.xlsx
@@ -40384,10 +40384,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010062D9CD9ACC6AE244981CDEFACE8F40CE" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5588035a854d9997c1d7df24985cfe90">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="433138c1-cfdf-4f6b-89e8-511447de8f15" xmlns:ns3="50b1dd69-4c56-4a1c-b3ce-7cd2bac560be" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08b0b5a8a4dc2a6a7064cc49017e9875" ns2:_="" ns3:_="">
-    <xsd:import namespace="433138c1-cfdf-4f6b-89e8-511447de8f15"/>
-    <xsd:import namespace="50b1dd69-4c56-4a1c-b3ce-7cd2bac560be"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C3FF88792079FE4CAD7BBDE0BC7B7482" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10b42e779589e082fc18e8126cc73c95">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5b833577-d5f3-4c92-a991-e0f5e5f065ff" xmlns:ns3="f82658c3-1dde-4375-8027-c01e071e8904" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="929128d0b677e760dca1e9118ba1563a" ns2:_="" ns3:_="">
+    <xsd:import namespace="5b833577-d5f3-4c92-a991-e0f5e5f065ff"/>
+    <xsd:import namespace="f82658c3-1dde-4375-8027-c01e071e8904"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -40396,16 +40396,18 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
@@ -40414,7 +40416,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="433138c1-cfdf-4f6b-89e8-511447de8f15" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5b833577-d5f3-4c92-a991-e0f5e5f065ff" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -40427,55 +40429,77 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceLocation" ma:index="12" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c10ff052-0d63-4843-8ea7-8646ee637017" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="191912c3-2eeb-460f-a7fe-a561d54f8fcf" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="21" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="50b1dd69-4c56-4a1c-b3ce-7cd2bac560be" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f82658c3-1dde-4375-8027-c01e071e8904" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b18b782b-ba8f-4525-ba6f-3696a66c0085}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="50b1dd69-4c56-4a1c-b3ce-7cd2bac560be">
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{6ad748f0-b28b-4f4f-b358-e143e647cf5a}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="f82658c3-1dde-4375-8027-c01e071e8904">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -40485,32 +40509,6 @@
           </xsd:extension>
         </xsd:complexContent>
       </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="19" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="20" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -40615,10 +40613,10 @@
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="433138c1-cfdf-4f6b-89e8-511447de8f15">
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5b833577-d5f3-4c92-a991-e0f5e5f065ff">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="50b1dd69-4c56-4a1c-b3ce-7cd2bac560be" xsi:nil="true"/>
+    <TaxCatchAll xmlns="f82658c3-1dde-4375-8027-c01e071e8904" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
@@ -40633,22 +40631,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88E36799-CA6B-4BDB-9F8A-B1B5CB126B31}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="433138c1-cfdf-4f6b-89e8-511447de8f15"/>
-    <ds:schemaRef ds:uri="50b1dd69-4c56-4a1c-b3ce-7cd2bac560be"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E74FE-DDD1-4B4B-8317-5BA2D272223D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>